<commit_message>
fix(LOG-029-F): saneamiento integral de XML eliminando conditionalFormatting en plantilla y generador para resolver error HRESULT 0x8000ffff en Excel
</commit_message>
<xml_diff>
--- a/templates/LOG-029-F.xlsx
+++ b/templates/LOG-029-F.xlsx
@@ -4191,12 +4191,6 @@
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="E12:F12"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D4">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D13">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I18:I27" xr:uid="{13C89437-37DB-4317-9CB4-8C6525EDDDF4}">
       <formula1>"SIN NOVEDAD, CON NOVEDAD"</formula1>
@@ -5967,9 +5961,6 @@
     <mergeCell ref="C125:C126"/>
     <mergeCell ref="A127:A128"/>
   </mergeCells>
-  <conditionalFormatting sqref="B117:B121 B107 B95 B37:B41 B1:B35 B43:B46 B65:B82 B86:B93 B123:B125 B127:B129 B159:B162">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7310,20 +7301,6 @@
     </row>
   </sheetData>
   <autoFilter ref="C1:F1" xr:uid="{B00816D2-9CAC-4A90-93E1-A5DE0272A7B6}"/>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F9">
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Serial no encontrado">
-      <formula>NOT(ISERROR(SEARCH("Serial no encontrado",F2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Serial Validado">
-      <formula>NOT(ISERROR(SEARCH("Serial Validado",F2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>